<commit_message>
update: implements CELL("filename") to return [WorkbookName.xlsx]SheetName
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/CELL.xlsx
+++ b/xlsx/tests/calc_tests/CELL.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E48B7A6C-4846-46F7-A13F-65F208757F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06FD819D-AC68-49C2-BBDE-035DCE73E477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CELL" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
   <si>
     <t>REFERENCE</t>
   </si>
@@ -110,9 +110,6 @@
     <t>Implicit intersection</t>
   </si>
   <si>
-    <t>filename</t>
-  </si>
-  <si>
     <t>format</t>
   </si>
   <si>
@@ -177,6 +174,24 @@
   </si>
   <si>
     <t>Invalid info type: blank</t>
+  </si>
+  <si>
+    <t>=CELL("format",A16)</t>
+  </si>
+  <si>
+    <t>=CELL("parentheses",A17)</t>
+  </si>
+  <si>
+    <t>=CELL("prefix",A18)</t>
+  </si>
+  <si>
+    <t>=CELL("protect",A19)</t>
+  </si>
+  <si>
+    <t>=CELL("color",A9)</t>
+  </si>
+  <si>
+    <t>=CELL("width",A32)</t>
   </si>
 </sst>
 </file>
@@ -187,7 +202,7 @@
     <numFmt numFmtId="164" formatCode="0.0000000000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -259,7 +274,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -282,6 +297,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,17 +586,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F54CD0-8216-4E1F-9732-2CE5FAC307BD}">
-  <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:L38"/>
+  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="2" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="53.140625" customWidth="1"/>
-    <col min="5" max="5" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.59765625" customWidth="1"/>
+    <col min="2" max="3" width="15.73046875" customWidth="1"/>
+    <col min="4" max="4" width="53.1328125" customWidth="1"/>
+    <col min="5" max="5" width="27.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75">
+    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -589,7 +610,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -605,7 +626,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -617,7 +638,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -632,7 +653,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
@@ -647,7 +668,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="30.75">
+    <row r="6" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" s="7">
         <v>3</v>
       </c>
@@ -661,7 +682,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>3</v>
       </c>
@@ -673,7 +694,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>4</v>
       </c>
@@ -688,13 +709,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="2" customFormat="1">
+    <row r="9" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B9" ca="1">CELL("color",A9)</f>
-        <v>#VALUE!</v>
+      <c r="B9" s="13" t="s">
+        <v>44</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -710,7 +730,7 @@
       <c r="K9"/>
       <c r="L9"/>
     </row>
-    <row r="10" spans="1:12" s="2" customFormat="1">
+    <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>3.4</v>
       </c>
@@ -729,7 +749,7 @@
       <c r="K10"/>
       <c r="L10"/>
     </row>
-    <row r="11" spans="1:12" s="2" customFormat="1">
+    <row r="11" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A11"/>
       <c r="B11" s="3" cm="1">
         <f t="array" aca="1" ref="B11" ca="1">CELL("contents",A11)</f>
@@ -749,7 +769,7 @@
       <c r="K11"/>
       <c r="L11"/>
     </row>
-    <row r="12" spans="1:12" s="2" customFormat="1">
+    <row r="12" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A12" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -772,7 +792,7 @@
       <c r="K12"/>
       <c r="L12"/>
     </row>
-    <row r="13" spans="1:12" s="2" customFormat="1">
+    <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A13" t="e">
         <f>NA()</f>
         <v>#N/A</v>
@@ -797,7 +817,7 @@
       <c r="K13"/>
       <c r="L13"/>
     </row>
-    <row r="14" spans="1:12" s="2" customFormat="1">
+    <row r="14" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>3</v>
       </c>
@@ -821,7 +841,7 @@
       <c r="K14"/>
       <c r="L14"/>
     </row>
-    <row r="15" spans="1:12" s="2" customFormat="1" ht="30.75">
+    <row r="15" spans="1:12" s="2" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A15" s="7"/>
       <c r="B15" s="11" t="s">
         <v>16</v>
@@ -842,37 +862,32 @@
       <c r="K15"/>
       <c r="L15"/>
     </row>
-    <row r="16" spans="1:12" s="2" customFormat="1">
+    <row r="16" spans="1:12" s="2" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16">
-        <v>4</v>
-      </c>
-      <c r="B16" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B16" ca="1">CELL("filename",A16)</f>
-        <v>#VALUE!</v>
+        <v>5</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="C16" t="s">
         <v>18</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E16"/>
-      <c r="F16">
-        <v>5</v>
-      </c>
       <c r="G16"/>
       <c r="H16"/>
       <c r="J16"/>
       <c r="K16"/>
       <c r="L16"/>
     </row>
-    <row r="17" spans="1:12" s="2" customFormat="1">
+    <row r="17" spans="1:12" s="2" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A17">
-        <v>5</v>
-      </c>
-      <c r="B17" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B17" ca="1">CELL("format",A17)</f>
-        <v>#VALUE!</v>
+        <v>6</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="C17" t="s">
         <v>19</v>
@@ -881,19 +896,19 @@
         <v>12</v>
       </c>
       <c r="E17"/>
+      <c r="F17"/>
       <c r="G17"/>
       <c r="H17"/>
       <c r="J17"/>
       <c r="K17"/>
       <c r="L17"/>
     </row>
-    <row r="18" spans="1:12" s="2" customFormat="1">
+    <row r="18" spans="1:12" s="2" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A18">
-        <v>6</v>
-      </c>
-      <c r="B18" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B18" ca="1">CELL("parentheses",A18)</f>
-        <v>#VALUE!</v>
+        <v>7</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
@@ -909,13 +924,12 @@
       <c r="K18"/>
       <c r="L18"/>
     </row>
-    <row r="19" spans="1:12" s="2" customFormat="1">
+    <row r="19" spans="1:12" s="2" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A19">
-        <v>7</v>
-      </c>
-      <c r="B19" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B19" ca="1">CELL("prefix",A19)</f>
-        <v>#VALUE!</v>
+        <v>8</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="C19" t="s">
         <v>21</v>
@@ -931,19 +945,16 @@
       <c r="K19"/>
       <c r="L19"/>
     </row>
-    <row r="20" spans="1:12" s="2" customFormat="1">
+    <row r="20" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A20">
-        <v>8</v>
-      </c>
-      <c r="B20" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B20" ca="1">CELL("protect",A20)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="3" cm="1">
+        <f t="array" aca="1" ref="B20" ca="1">CELL("row",A20)</f>
+        <v>20</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -953,16 +964,19 @@
       <c r="K20"/>
       <c r="L20"/>
     </row>
-    <row r="21" spans="1:12" s="2" customFormat="1">
+    <row r="21" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A21">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B21" s="3" cm="1">
-        <f t="array" aca="1" ref="B21" ca="1">CELL("row",A21)</f>
-        <v>21</v>
+        <f t="array" aca="1" ref="B21" ca="1">CELL("row",A11:A21)</f>
+        <v>11</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
       </c>
       <c r="E21"/>
       <c r="F21"/>
@@ -972,19 +986,16 @@
       <c r="K21"/>
       <c r="L21"/>
     </row>
-    <row r="22" spans="1:12" s="2" customFormat="1">
+    <row r="22" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>10</v>
       </c>
-      <c r="B22" s="3" cm="1">
-        <f t="array" aca="1" ref="B22" ca="1">CELL("row",A11:A22)</f>
-        <v>11</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="B22" s="6" t="str" cm="1">
+        <f t="array" aca="1" ref="B22" ca="1">CELL("type",A22)</f>
+        <v>v</v>
+      </c>
+      <c r="C22" t="s">
         <v>23</v>
-      </c>
-      <c r="D22" t="s">
-        <v>6</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -994,16 +1005,17 @@
       <c r="K22"/>
       <c r="L22"/>
     </row>
-    <row r="23" spans="1:12" s="2" customFormat="1">
-      <c r="A23">
-        <v>10</v>
-      </c>
+    <row r="23" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A23"/>
       <c r="B23" s="6" t="str" cm="1">
         <f t="array" aca="1" ref="B23" ca="1">CELL("type",A23)</f>
-        <v>v</v>
+        <v>b</v>
       </c>
       <c r="C23" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="E23"/>
       <c r="F23"/>
@@ -1013,227 +1025,206 @@
       <c r="K23"/>
       <c r="L23"/>
     </row>
-    <row r="24" spans="1:12" s="2" customFormat="1">
-      <c r="A24"/>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
       <c r="B24" s="6" t="str" cm="1">
         <f t="array" aca="1" ref="B24" ca="1">CELL("type",A24)</f>
-        <v>b</v>
+        <v>l</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
-      <c r="J24"/>
-      <c r="K24"/>
-      <c r="L24"/>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A25" t="b">
+        <v>1</v>
       </c>
       <c r="B25" s="6" t="str" cm="1">
         <f t="array" aca="1" ref="B25" ca="1">CELL("type",A25)</f>
-        <v>l</v>
+        <v>v</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
-      <c r="A26" t="b">
-        <v>1</v>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A26">
+        <v>0</v>
       </c>
       <c r="B26" s="6" t="str" cm="1">
         <f t="array" aca="1" ref="B26" ca="1">CELL("type",A26)</f>
         <v>v</v>
       </c>
       <c r="C26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>0</v>
       </c>
       <c r="B27" s="6" t="str" cm="1">
-        <f t="array" aca="1" ref="B27" ca="1">CELL("type",A27)</f>
+        <f t="array" aca="1" ref="B27" ca="1">CELL("TYPE",A27)</f>
         <v>v</v>
       </c>
       <c r="C27" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
-      <c r="A28">
-        <v>0</v>
-      </c>
-      <c r="B28" s="6" t="str" cm="1">
-        <f t="array" aca="1" ref="B28" ca="1">CELL("TYPE",A28)</f>
-        <v>v</v>
-      </c>
-      <c r="C28" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
-      <c r="A29" t="e">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A28" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
+      </c>
+      <c r="B28" s="6" t="str" cm="1">
+        <f t="array" aca="1" ref="B28" ca="1">CELL("type",A28)</f>
+        <v>v</v>
+      </c>
+      <c r="C28" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A29" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
       </c>
       <c r="B29" s="6" t="str" cm="1">
         <f t="array" aca="1" ref="B29" ca="1">CELL("type",A29)</f>
         <v>v</v>
       </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
-      <c r="A30" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A30">
+        <v>2</v>
       </c>
       <c r="B30" s="6" t="str" cm="1">
-        <f t="array" aca="1" ref="B30" ca="1">CELL("type",A30)</f>
-        <v>v</v>
+        <f t="array" aca="1" ref="B30" ca="1">CELL("type", INDIRECT("A"&amp;10^6))</f>
+        <v>b</v>
       </c>
       <c r="C30" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12">
-      <c r="A31">
-        <v>2</v>
-      </c>
-      <c r="B31" s="6" t="str" cm="1">
-        <f t="array" aca="1" ref="B31" ca="1">CELL("type", INDIRECT("A"&amp;10^6))</f>
-        <v>b</v>
-      </c>
-      <c r="C31" t="s">
-        <v>24</v>
-      </c>
-      <c r="D31" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A31" s="7">
+        <v>3</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" ht="45.75">
-      <c r="A32" s="7">
-        <v>3</v>
-      </c>
-      <c r="B32" s="10" t="s">
+      <c r="C31" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D32" s="9" t="s">
+    </row>
+    <row r="32" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A32">
+        <v>13</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C32" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33">
-        <v>13</v>
+      <c r="D32" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>33</v>
       </c>
       <c r="B33" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B33" ca="1">CELL("width",A33)</f>
+        <f t="array" aca="1" ref="B33" ca="1">CELL(A33,A33)</f>
         <v>#VALUE!</v>
       </c>
       <c r="C33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B34" s="6" t="e" cm="1">
+        <f t="array" aca="1" ref="B34" ca="1">CELL("hello")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C34" t="s">
         <v>34</v>
-      </c>
-      <c r="B34" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B34" ca="1">CELL(A34,A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C34" t="s">
-        <v>35</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B35" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B35" ca="1">CELL("hello")</f>
+        <f t="array" aca="1" ref="B35" ca="1">CELL(TRUE)</f>
         <v>#VALUE!</v>
       </c>
       <c r="C35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B36" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B36" ca="1">CELL(TRUE)</f>
+        <f t="array" aca="1" ref="B36" ca="1">CELL(2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="C36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B37" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B37" ca="1">CELL(2)</f>
+        <f t="array" aca="1" ref="B37" ca="1">CELL("")</f>
         <v>#VALUE!</v>
       </c>
       <c r="C37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
-      <c r="B38" s="6" t="e" cm="1">
-        <f t="array" aca="1" ref="B38" ca="1">CELL("")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C38" t="s">
-        <v>35</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="4"/>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A38" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1244,7 +1235,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F019826-82F7-4B96-AB22-783A55CB1B8D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>